<commit_message>
updated spreadsheet generator to handle extra fields
</commit_message>
<xml_diff>
--- a/data/ejc-data-template-static-backup.xlsx
+++ b/data/ejc-data-template-static-backup.xlsx
@@ -32,7 +32,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Warren" sheetId="23" state="visible" r:id="rId23"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legend" sheetId="24" state="visible" r:id="rId24"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Data'!$A$2:$AU$602</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -40161,6 +40163,7 @@
       <c r="AU566" s="26" t="inlineStr"/>
     </row>
   </sheetData>
+  <autoFilter ref="A2:AU602"/>
   <mergeCells count="10">
     <mergeCell ref="I1:J1"/>
     <mergeCell ref="A1:D1"/>

</xml_diff>